<commit_message>
solved image upload bug
</commit_message>
<xml_diff>
--- a/data/proxies/good_proxies.xlsx
+++ b/data/proxies/good_proxies.xlsx
@@ -566,7 +566,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>3452.8</v>
+        <v>3724.6</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -580,7 +580,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-04-03 10:48:03 UTC</t>
+          <t>2026-04-06 08:58:53 UTC</t>
         </is>
       </c>
     </row>
@@ -591,7 +591,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>430.2</v>
+        <v>431</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -605,7 +605,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-04-06 07:15:13 UTC</t>
+          <t>2026-04-06 09:25:37 UTC</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>486.7</v>
+        <v>562.9</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -630,7 +630,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-04-06 07:13:50 UTC</t>
+          <t>2026-04-06 09:25:37 UTC</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>381.9</v>
+        <v>632.8</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -655,7 +655,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-04-06 07:15:13 UTC</t>
+          <t>2026-04-06 09:25:37 UTC</t>
         </is>
       </c>
     </row>
@@ -741,7 +741,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>217.2</v>
+        <v>274.5</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -755,7 +755,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-04-06 07:15:13 UTC</t>
+          <t>2026-04-06 09:25:37 UTC</t>
         </is>
       </c>
     </row>
@@ -766,7 +766,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>538</v>
+        <v>577.2</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -780,7 +780,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-04-06 07:15:13 UTC</t>
+          <t>2026-04-06 09:25:37 UTC</t>
         </is>
       </c>
     </row>
@@ -791,7 +791,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>308.1</v>
+        <v>410.6</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -805,7 +805,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-04-06 07:15:13 UTC</t>
+          <t>2026-04-06 09:25:37 UTC</t>
         </is>
       </c>
     </row>
@@ -816,7 +816,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1327.2</v>
+        <v>1283.9</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -830,7 +830,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026-04-03 10:55:03 UTC</t>
+          <t>2026-04-06 07:40:26 UTC</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>2476.6</v>
+        <v>3445.7</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -855,7 +855,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2026-04-03 10:55:03 UTC</t>
+          <t>2026-04-06 07:22:33 UTC</t>
         </is>
       </c>
     </row>
@@ -866,7 +866,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>3451.1</v>
+        <v>3471.2</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -880,7 +880,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2026-04-06 06:37:12 UTC</t>
+          <t>2026-04-06 07:44:18 UTC</t>
         </is>
       </c>
     </row>
@@ -961,7 +961,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>3296.2</v>
+        <v>3282.9</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -970,7 +970,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2026-04-06 07:12:33 UTC</t>
+          <t>2026-04-06 07:16:31 UTC</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>573.1</v>
+        <v>1038.2</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1010,7 +1010,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026-04-06 07:15:13 UTC</t>
+          <t>2026-04-06 09:25:37 UTC</t>
         </is>
       </c>
     </row>
@@ -1021,7 +1021,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>2376</v>
+        <v>947.3</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1030,7 +1030,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2026-04-03 11:15:42 UTC</t>
+          <t>2026-04-06 09:19:02 UTC</t>
         </is>
       </c>
     </row>
@@ -1041,7 +1041,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>966.7</v>
+        <v>761.2</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -1050,7 +1050,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2026-04-06 07:15:13 UTC</t>
+          <t>2026-04-06 08:45:32 UTC</t>
         </is>
       </c>
     </row>
@@ -1081,7 +1081,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>220.6</v>
+        <v>306.7</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -1090,7 +1090,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2026-04-06 07:15:13 UTC</t>
+          <t>2026-04-06 09:25:37 UTC</t>
         </is>
       </c>
     </row>
@@ -1101,7 +1101,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>1774.7</v>
+        <v>1588.4</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1110,7 +1110,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2026-04-03 11:18:09 UTC</t>
+          <t>2026-04-06 08:55:43 UTC</t>
         </is>
       </c>
     </row>
@@ -1141,7 +1141,7 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>3338.6</v>
+        <v>2579.1</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1150,7 +1150,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2026-04-03 11:18:29 UTC</t>
+          <t>2026-04-06 07:44:18 UTC</t>
         </is>
       </c>
     </row>
@@ -1161,7 +1161,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>4524.4</v>
+        <v>1202.2</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1170,7 +1170,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2026-04-03 11:20:57 UTC</t>
+          <t>2026-04-06 09:11:31 UTC</t>
         </is>
       </c>
     </row>
@@ -1221,7 +1221,7 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>5144.9</v>
+        <v>1305.8</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -1230,7 +1230,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2026-04-03 11:21:37 UTC</t>
+          <t>2026-04-06 09:05:57 UTC</t>
         </is>
       </c>
     </row>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>3883.3</v>
+        <v>1859.3</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -1250,7 +1250,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2026-04-06 07:13:50 UTC</t>
+          <t>2026-04-06 08:35:17 UTC</t>
         </is>
       </c>
     </row>
@@ -1261,7 +1261,7 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>1452.1</v>
+        <v>247.7</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1270,7 +1270,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>2026-04-03 11:21:37 UTC</t>
+          <t>2026-04-06 09:20:18 UTC</t>
         </is>
       </c>
     </row>
@@ -1301,7 +1301,7 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>4793.6</v>
+        <v>1241.6</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1310,7 +1310,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>2026-04-03 11:22:22 UTC</t>
+          <t>2026-04-06 09:11:31 UTC</t>
         </is>
       </c>
     </row>
@@ -1341,7 +1341,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>3348.5</v>
+        <v>1419</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1350,7 +1350,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>2026-04-03 11:22:22 UTC</t>
+          <t>2026-04-06 08:38:29 UTC</t>
         </is>
       </c>
     </row>
@@ -1361,7 +1361,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>2688.5</v>
+        <v>3474.1</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -1370,7 +1370,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>2026-04-03 11:22:22 UTC</t>
+          <t>2026-04-06 07:47:05 UTC</t>
         </is>
       </c>
     </row>
@@ -1381,7 +1381,7 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>4062.9</v>
+        <v>311</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -1390,7 +1390,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>2026-04-03 11:22:22 UTC</t>
+          <t>2026-04-06 07:55:52 UTC</t>
         </is>
       </c>
     </row>
@@ -1401,7 +1401,7 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>5517.7</v>
+        <v>1443.2</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1410,7 +1410,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>2026-04-03 11:22:22 UTC</t>
+          <t>2026-04-06 09:19:02 UTC</t>
         </is>
       </c>
     </row>
@@ -1421,7 +1421,7 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>5629.3</v>
+        <v>1366.1</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1430,7 +1430,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>2026-04-03 11:22:22 UTC</t>
+          <t>2026-04-06 08:33:36 UTC</t>
         </is>
       </c>
     </row>
@@ -1461,7 +1461,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>5485.1</v>
+        <v>2033.2</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -1470,7 +1470,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>2026-04-03 11:22:55 UTC</t>
+          <t>2026-04-06 08:41:44 UTC</t>
         </is>
       </c>
     </row>
@@ -1501,7 +1501,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>2824.4</v>
+        <v>3288.1</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -1510,7 +1510,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>2026-04-03 11:30:47 UTC</t>
+          <t>2026-04-06 08:52:00 UTC</t>
         </is>
       </c>
     </row>
@@ -1521,7 +1521,7 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>1014.4</v>
+        <v>580</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
@@ -1530,7 +1530,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>2026-04-06 06:58:37 UTC</t>
+          <t>2026-04-06 09:25:37 UTC</t>
         </is>
       </c>
     </row>
@@ -1541,7 +1541,7 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>859.6</v>
+        <v>900.5</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
@@ -1550,7 +1550,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>2026-04-06 07:15:13 UTC</t>
+          <t>2026-04-06 09:11:31 UTC</t>
         </is>
       </c>
     </row>
@@ -1561,7 +1561,7 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>3078</v>
+        <v>1290.5</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
@@ -1570,7 +1570,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>2026-04-03 11:30:47 UTC</t>
+          <t>2026-04-06 08:35:17 UTC</t>
         </is>
       </c>
     </row>
@@ -1621,7 +1621,7 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>5343.8</v>
+        <v>3422.9</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
@@ -1630,7 +1630,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>2026-04-03 11:31:45 UTC</t>
+          <t>2026-04-06 09:04:14 UTC</t>
         </is>
       </c>
     </row>
@@ -1661,7 +1661,7 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>2591.5</v>
+        <v>1667.4</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
@@ -1670,7 +1670,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>2026-04-03 11:35:08 UTC</t>
+          <t>2026-04-06 09:25:37 UTC</t>
         </is>
       </c>
     </row>
@@ -1781,7 +1781,7 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>1741.7</v>
+        <v>1346.2</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
@@ -1790,7 +1790,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>2026-04-03 11:36:22 UTC</t>
+          <t>2026-04-06 07:48:23 UTC</t>
         </is>
       </c>
     </row>
@@ -2701,7 +2701,7 @@
         </is>
       </c>
       <c r="B109" t="n">
-        <v>418.7</v>
+        <v>4363.6</v>
       </c>
       <c r="C109" t="inlineStr">
         <is>
@@ -2710,7 +2710,7 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>2026-04-06 07:12:33 UTC</t>
+          <t>2026-04-06 09:05:57 UTC</t>
         </is>
       </c>
     </row>
@@ -2721,7 +2721,7 @@
         </is>
       </c>
       <c r="B110" t="n">
-        <v>4703.5</v>
+        <v>233.7</v>
       </c>
       <c r="C110" t="inlineStr">
         <is>
@@ -2730,7 +2730,7 @@
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>2026-04-06 07:15:13 UTC</t>
+          <t>2026-04-06 09:24:07 UTC</t>
         </is>
       </c>
     </row>
@@ -2741,7 +2741,7 @@
         </is>
       </c>
       <c r="B111" t="n">
-        <v>3466</v>
+        <v>1342.9</v>
       </c>
       <c r="C111" t="inlineStr">
         <is>
@@ -2750,7 +2750,7 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>2026-04-05 10:06:45 UTC</t>
+          <t>2026-04-06 09:17:46 UTC</t>
         </is>
       </c>
     </row>
@@ -2781,7 +2781,7 @@
         </is>
       </c>
       <c r="B113" t="n">
-        <v>2287.1</v>
+        <v>1118</v>
       </c>
       <c r="C113" t="inlineStr">
         <is>
@@ -2790,7 +2790,7 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>2026-04-05 10:09:16 UTC</t>
+          <t>2026-04-06 08:12:59 UTC</t>
         </is>
       </c>
     </row>
@@ -2801,7 +2801,7 @@
         </is>
       </c>
       <c r="B114" t="n">
-        <v>2141.3</v>
+        <v>2011.3</v>
       </c>
       <c r="C114" t="inlineStr">
         <is>
@@ -2810,7 +2810,7 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>2026-04-05 10:09:16 UTC</t>
+          <t>2026-04-06 09:25:37 UTC</t>
         </is>
       </c>
     </row>
@@ -2821,7 +2821,7 @@
         </is>
       </c>
       <c r="B115" t="n">
-        <v>2546</v>
+        <v>1492.4</v>
       </c>
       <c r="C115" t="inlineStr">
         <is>
@@ -2830,7 +2830,7 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>2026-04-05 10:09:16 UTC</t>
+          <t>2026-04-06 08:04:33 UTC</t>
         </is>
       </c>
     </row>
@@ -2841,7 +2841,7 @@
         </is>
       </c>
       <c r="B116" t="n">
-        <v>2230.2</v>
+        <v>2627.2</v>
       </c>
       <c r="C116" t="inlineStr">
         <is>
@@ -2850,7 +2850,7 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>2026-04-06 07:15:13 UTC</t>
+          <t>2026-04-06 09:25:37 UTC</t>
         </is>
       </c>
     </row>
@@ -2861,7 +2861,7 @@
         </is>
       </c>
       <c r="B117" t="n">
-        <v>2322.9</v>
+        <v>906.7</v>
       </c>
       <c r="C117" t="inlineStr">
         <is>
@@ -2870,7 +2870,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>2026-04-05 10:10:37 UTC</t>
+          <t>2026-04-06 09:24:07 UTC</t>
         </is>
       </c>
     </row>
@@ -2921,7 +2921,7 @@
         </is>
       </c>
       <c r="B120" t="n">
-        <v>14.1</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="C120" t="inlineStr">
         <is>
@@ -2930,7 +2930,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>2026-04-06 06:57:06 UTC</t>
+          <t>2026-04-06 09:09:56 UTC</t>
         </is>
       </c>
     </row>
@@ -2961,7 +2961,7 @@
         </is>
       </c>
       <c r="B122" t="n">
-        <v>150.2</v>
+        <v>131.9</v>
       </c>
       <c r="C122" t="inlineStr">
         <is>
@@ -2970,7 +2970,7 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>2026-04-06 06:57:06 UTC</t>
+          <t>2026-04-06 09:09:56 UTC</t>
         </is>
       </c>
     </row>
@@ -3061,7 +3061,7 @@
         </is>
       </c>
       <c r="B127" t="n">
-        <v>231.4</v>
+        <v>186.3</v>
       </c>
       <c r="C127" t="inlineStr">
         <is>
@@ -3070,7 +3070,7 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>2026-04-06 06:58:37 UTC</t>
+          <t>2026-04-06 09:09:56 UTC</t>
         </is>
       </c>
     </row>
@@ -3141,7 +3141,7 @@
         </is>
       </c>
       <c r="B131" t="n">
-        <v>198.4</v>
+        <v>329.1</v>
       </c>
       <c r="C131" t="inlineStr">
         <is>
@@ -3150,7 +3150,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>2026-04-06 06:57:06 UTC</t>
+          <t>2026-04-06 09:09:56 UTC</t>
         </is>
       </c>
     </row>
@@ -3161,7 +3161,7 @@
         </is>
       </c>
       <c r="B132" t="n">
-        <v>252.7</v>
+        <v>275.8</v>
       </c>
       <c r="C132" t="inlineStr">
         <is>
@@ -3170,7 +3170,7 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>2026-04-05 10:10:37 UTC</t>
+          <t>2026-04-06 09:08:54 UTC</t>
         </is>
       </c>
     </row>
@@ -3241,7 +3241,7 @@
         </is>
       </c>
       <c r="B136" t="n">
-        <v>254.3</v>
+        <v>3412.6</v>
       </c>
       <c r="C136" t="inlineStr">
         <is>
@@ -3250,7 +3250,7 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>2026-04-05 10:10:37 UTC</t>
+          <t>2026-04-06 09:15:11 UTC</t>
         </is>
       </c>
     </row>
@@ -3841,7 +3841,7 @@
         </is>
       </c>
       <c r="B166" t="n">
-        <v>1999.3</v>
+        <v>803.2</v>
       </c>
       <c r="C166" t="inlineStr">
         <is>
@@ -3850,7 +3850,7 @@
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>2026-04-06 06:34:49 UTC</t>
+          <t>2026-04-06 08:03:11 UTC</t>
         </is>
       </c>
     </row>
@@ -3961,7 +3961,7 @@
         </is>
       </c>
       <c r="B172" t="n">
-        <v>1069.6</v>
+        <v>1056.4</v>
       </c>
       <c r="C172" t="inlineStr">
         <is>
@@ -3970,7 +3970,7 @@
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>2026-04-06 07:15:13 UTC</t>
+          <t>2026-04-06 07:40:26 UTC</t>
         </is>
       </c>
     </row>
@@ -4301,7 +4301,7 @@
         </is>
       </c>
       <c r="B189" t="n">
-        <v>235.1</v>
+        <v>172.1</v>
       </c>
       <c r="C189" t="inlineStr">
         <is>
@@ -4310,7 +4310,7 @@
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>2026-04-05 10:11:03 UTC</t>
+          <t>2026-04-06 09:09:56 UTC</t>
         </is>
       </c>
     </row>
@@ -4321,7 +4321,7 @@
         </is>
       </c>
       <c r="B190" t="n">
-        <v>251.1</v>
+        <v>281.3</v>
       </c>
       <c r="C190" t="inlineStr">
         <is>
@@ -4330,7 +4330,7 @@
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>2026-04-05 10:11:03 UTC</t>
+          <t>2026-04-06 09:08:54 UTC</t>
         </is>
       </c>
     </row>
@@ -4361,7 +4361,7 @@
         </is>
       </c>
       <c r="B192" t="n">
-        <v>252.4</v>
+        <v>204.6</v>
       </c>
       <c r="C192" t="inlineStr">
         <is>
@@ -4370,7 +4370,7 @@
       </c>
       <c r="E192" t="inlineStr">
         <is>
-          <t>2026-04-05 10:11:03 UTC</t>
+          <t>2026-04-06 09:25:37 UTC</t>
         </is>
       </c>
     </row>
@@ -4561,7 +4561,7 @@
         </is>
       </c>
       <c r="B202" t="n">
-        <v>251.1</v>
+        <v>280.8</v>
       </c>
       <c r="C202" t="inlineStr">
         <is>
@@ -4570,7 +4570,7 @@
       </c>
       <c r="E202" t="inlineStr">
         <is>
-          <t>2026-04-05 10:11:03 UTC</t>
+          <t>2026-04-06 09:08:54 UTC</t>
         </is>
       </c>
     </row>
@@ -4621,7 +4621,7 @@
         </is>
       </c>
       <c r="B205" t="n">
-        <v>529.8</v>
+        <v>590.2</v>
       </c>
       <c r="C205" t="inlineStr">
         <is>
@@ -4630,7 +4630,7 @@
       </c>
       <c r="E205" t="inlineStr">
         <is>
-          <t>2026-04-06 07:15:13 UTC</t>
+          <t>2026-04-06 09:25:37 UTC</t>
         </is>
       </c>
     </row>
@@ -5121,7 +5121,7 @@
         </is>
       </c>
       <c r="B230" t="n">
-        <v>253</v>
+        <v>299.4</v>
       </c>
       <c r="C230" t="inlineStr">
         <is>
@@ -5130,7 +5130,7 @@
       </c>
       <c r="E230" t="inlineStr">
         <is>
-          <t>2026-04-05 10:11:03 UTC</t>
+          <t>2026-04-06 09:25:37 UTC</t>
         </is>
       </c>
     </row>
@@ -5601,7 +5601,7 @@
         </is>
       </c>
       <c r="B254" t="n">
-        <v>154.4</v>
+        <v>274.3</v>
       </c>
       <c r="C254" t="inlineStr">
         <is>
@@ -5610,7 +5610,7 @@
       </c>
       <c r="E254" t="inlineStr">
         <is>
-          <t>2026-04-06 06:58:37 UTC</t>
+          <t>2026-04-06 09:25:37 UTC</t>
         </is>
       </c>
     </row>
@@ -5741,7 +5741,7 @@
         </is>
       </c>
       <c r="B261" t="n">
-        <v>363.5</v>
+        <v>286.3</v>
       </c>
       <c r="C261" t="inlineStr">
         <is>
@@ -5750,7 +5750,7 @@
       </c>
       <c r="E261" t="inlineStr">
         <is>
-          <t>2026-04-06 07:15:13 UTC</t>
+          <t>2026-04-06 09:25:37 UTC</t>
         </is>
       </c>
     </row>
@@ -5761,7 +5761,7 @@
         </is>
       </c>
       <c r="B262" t="n">
-        <v>1859.7</v>
+        <v>934.8</v>
       </c>
       <c r="C262" t="inlineStr">
         <is>
@@ -5770,7 +5770,7 @@
       </c>
       <c r="E262" t="inlineStr">
         <is>
-          <t>2026-04-06 07:15:13 UTC</t>
+          <t>2026-04-06 09:08:54 UTC</t>
         </is>
       </c>
     </row>
@@ -5841,7 +5841,7 @@
         </is>
       </c>
       <c r="B266" t="n">
-        <v>60.8</v>
+        <v>55.6</v>
       </c>
       <c r="C266" t="inlineStr">
         <is>
@@ -5850,7 +5850,7 @@
       </c>
       <c r="E266" t="inlineStr">
         <is>
-          <t>2026-04-06 06:57:06 UTC</t>
+          <t>2026-04-06 09:09:56 UTC</t>
         </is>
       </c>
     </row>
@@ -5881,7 +5881,7 @@
         </is>
       </c>
       <c r="B268" t="n">
-        <v>221.7</v>
+        <v>217.2</v>
       </c>
       <c r="C268" t="inlineStr">
         <is>
@@ -5890,7 +5890,7 @@
       </c>
       <c r="E268" t="inlineStr">
         <is>
-          <t>2026-04-06 06:57:06 UTC</t>
+          <t>2026-04-06 09:09:56 UTC</t>
         </is>
       </c>
     </row>
@@ -6041,7 +6041,7 @@
         </is>
       </c>
       <c r="B276" t="n">
-        <v>4584</v>
+        <v>2530.6</v>
       </c>
       <c r="C276" t="inlineStr">
         <is>
@@ -6050,7 +6050,7 @@
       </c>
       <c r="E276" t="inlineStr">
         <is>
-          <t>2026-04-05 10:17:35 UTC</t>
+          <t>2026-04-06 09:22:38 UTC</t>
         </is>
       </c>
     </row>
@@ -6721,7 +6721,7 @@
         </is>
       </c>
       <c r="B310" t="n">
-        <v>217.7</v>
+        <v>1249.8</v>
       </c>
       <c r="C310" t="inlineStr">
         <is>
@@ -6730,7 +6730,7 @@
       </c>
       <c r="E310" t="inlineStr">
         <is>
-          <t>2026-04-06 07:15:13 UTC</t>
+          <t>2026-04-06 07:17:51 UTC</t>
         </is>
       </c>
     </row>
@@ -7921,7 +7921,7 @@
         </is>
       </c>
       <c r="B370" t="n">
-        <v>238.8</v>
+        <v>3226.3</v>
       </c>
       <c r="C370" t="inlineStr">
         <is>
@@ -7930,7 +7930,7 @@
       </c>
       <c r="E370" t="inlineStr">
         <is>
-          <t>2026-04-05 10:21:20 UTC</t>
+          <t>2026-04-06 09:07:33 UTC</t>
         </is>
       </c>
     </row>
@@ -8341,7 +8341,7 @@
         </is>
       </c>
       <c r="B391" t="n">
-        <v>232.1</v>
+        <v>232.3</v>
       </c>
       <c r="C391" t="inlineStr">
         <is>
@@ -8350,7 +8350,7 @@
       </c>
       <c r="E391" t="inlineStr">
         <is>
-          <t>2026-04-05 10:21:20 UTC</t>
+          <t>2026-04-06 09:25:37 UTC</t>
         </is>
       </c>
     </row>
@@ -9461,7 +9461,7 @@
         </is>
       </c>
       <c r="B447" t="n">
-        <v>2658.4</v>
+        <v>3476.5</v>
       </c>
       <c r="C447" t="inlineStr">
         <is>
@@ -9470,7 +9470,7 @@
       </c>
       <c r="E447" t="inlineStr">
         <is>
-          <t>2026-04-05 10:21:20 UTC</t>
+          <t>2026-04-06 07:34:05 UTC</t>
         </is>
       </c>
     </row>
@@ -9701,7 +9701,7 @@
         </is>
       </c>
       <c r="B459" t="n">
-        <v>1655.4</v>
+        <v>3505.1</v>
       </c>
       <c r="C459" t="inlineStr">
         <is>
@@ -9710,7 +9710,7 @@
       </c>
       <c r="E459" t="inlineStr">
         <is>
-          <t>2026-04-05 10:28:03 UTC</t>
+          <t>2026-04-06 09:19:02 UTC</t>
         </is>
       </c>
     </row>
@@ -9741,7 +9741,7 @@
         </is>
       </c>
       <c r="B461" t="n">
-        <v>1544.5</v>
+        <v>4118.6</v>
       </c>
       <c r="C461" t="inlineStr">
         <is>
@@ -9750,7 +9750,7 @@
       </c>
       <c r="E461" t="inlineStr">
         <is>
-          <t>2026-04-06 07:15:13 UTC</t>
+          <t>2026-04-06 08:55:43 UTC</t>
         </is>
       </c>
     </row>
@@ -9801,7 +9801,7 @@
         </is>
       </c>
       <c r="B464" t="n">
-        <v>3266.3</v>
+        <v>1218.7</v>
       </c>
       <c r="C464" t="inlineStr">
         <is>
@@ -9810,7 +9810,7 @@
       </c>
       <c r="E464" t="inlineStr">
         <is>
-          <t>2026-04-06 06:58:37 UTC</t>
+          <t>2026-04-06 07:16:31 UTC</t>
         </is>
       </c>
     </row>
@@ -10041,7 +10041,7 @@
         </is>
       </c>
       <c r="B476" t="n">
-        <v>3558</v>
+        <v>1418</v>
       </c>
       <c r="C476" t="inlineStr">
         <is>
@@ -10050,7 +10050,7 @@
       </c>
       <c r="E476" t="inlineStr">
         <is>
-          <t>2026-04-05 10:29:46 UTC</t>
+          <t>2026-04-06 09:24:07 UTC</t>
         </is>
       </c>
     </row>
@@ -10081,7 +10081,7 @@
         </is>
       </c>
       <c r="B478" t="n">
-        <v>2336.7</v>
+        <v>1605.1</v>
       </c>
       <c r="C478" t="inlineStr">
         <is>
@@ -10090,7 +10090,7 @@
       </c>
       <c r="E478" t="inlineStr">
         <is>
-          <t>2026-04-06 07:12:33 UTC</t>
+          <t>2026-04-06 08:41:44 UTC</t>
         </is>
       </c>
     </row>
@@ -10121,7 +10121,7 @@
         </is>
       </c>
       <c r="B480" t="n">
-        <v>642.2</v>
+        <v>916.5</v>
       </c>
       <c r="C480" t="inlineStr">
         <is>
@@ -10130,7 +10130,7 @@
       </c>
       <c r="E480" t="inlineStr">
         <is>
-          <t>2026-04-06 07:15:13 UTC</t>
+          <t>2026-04-06 09:24:07 UTC</t>
         </is>
       </c>
     </row>
@@ -10161,7 +10161,7 @@
         </is>
       </c>
       <c r="B482" t="n">
-        <v>3488.6</v>
+        <v>199.4</v>
       </c>
       <c r="C482" t="inlineStr">
         <is>
@@ -10170,7 +10170,7 @@
       </c>
       <c r="E482" t="inlineStr">
         <is>
-          <t>2026-04-05 10:36:49 UTC</t>
+          <t>2026-04-06 09:17:46 UTC</t>
         </is>
       </c>
     </row>
@@ -10181,7 +10181,7 @@
         </is>
       </c>
       <c r="B483" t="n">
-        <v>2937.9</v>
+        <v>3840.9</v>
       </c>
       <c r="C483" t="inlineStr">
         <is>
@@ -10190,7 +10190,7 @@
       </c>
       <c r="E483" t="inlineStr">
         <is>
-          <t>2026-04-05 10:36:49 UTC</t>
+          <t>2026-04-06 09:25:37 UTC</t>
         </is>
       </c>
     </row>
@@ -10241,7 +10241,7 @@
         </is>
       </c>
       <c r="B486" t="n">
-        <v>2782.5</v>
+        <v>1160.8</v>
       </c>
       <c r="C486" t="inlineStr">
         <is>
@@ -10250,7 +10250,7 @@
       </c>
       <c r="E486" t="inlineStr">
         <is>
-          <t>2026-04-05 10:37:33 UTC</t>
+          <t>2026-04-06 09:19:02 UTC</t>
         </is>
       </c>
     </row>
@@ -10381,7 +10381,7 @@
         </is>
       </c>
       <c r="B493" t="n">
-        <v>241.5</v>
+        <v>394.1</v>
       </c>
       <c r="C493" t="inlineStr">
         <is>
@@ -10390,7 +10390,7 @@
       </c>
       <c r="E493" t="inlineStr">
         <is>
-          <t>2026-04-05 10:48:24 UTC</t>
+          <t>2026-04-06 09:08:54 UTC</t>
         </is>
       </c>
     </row>
@@ -10481,7 +10481,7 @@
         </is>
       </c>
       <c r="B498" t="n">
-        <v>4574.3</v>
+        <v>283.3</v>
       </c>
       <c r="C498" t="inlineStr">
         <is>
@@ -10490,7 +10490,7 @@
       </c>
       <c r="E498" t="inlineStr">
         <is>
-          <t>2026-04-05 10:55:03 UTC</t>
+          <t>2026-04-06 07:38:07 UTC</t>
         </is>
       </c>
     </row>
@@ -10501,7 +10501,7 @@
         </is>
       </c>
       <c r="B499" t="n">
-        <v>3086.7</v>
+        <v>854.6</v>
       </c>
       <c r="C499" t="inlineStr">
         <is>
@@ -10510,7 +10510,7 @@
       </c>
       <c r="E499" t="inlineStr">
         <is>
-          <t>2026-04-05 10:56:03 UTC</t>
+          <t>2026-04-06 07:36:49 UTC</t>
         </is>
       </c>
     </row>
@@ -10521,7 +10521,7 @@
         </is>
       </c>
       <c r="B500" t="n">
-        <v>2338.8</v>
+        <v>733.8</v>
       </c>
       <c r="C500" t="inlineStr">
         <is>
@@ -10530,7 +10530,7 @@
       </c>
       <c r="E500" t="inlineStr">
         <is>
-          <t>2026-04-05 10:56:03 UTC</t>
+          <t>2026-04-06 08:07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -10541,7 +10541,7 @@
         </is>
       </c>
       <c r="B501" t="n">
-        <v>3846.4</v>
+        <v>916.7</v>
       </c>
       <c r="C501" t="inlineStr">
         <is>
@@ -10550,7 +10550,7 @@
       </c>
       <c r="E501" t="inlineStr">
         <is>
-          <t>2026-04-05 10:56:03 UTC</t>
+          <t>2026-04-06 09:22:38 UTC</t>
         </is>
       </c>
     </row>
@@ -10561,7 +10561,7 @@
         </is>
       </c>
       <c r="B502" t="n">
-        <v>2209.7</v>
+        <v>777.6</v>
       </c>
       <c r="C502" t="inlineStr">
         <is>
@@ -10570,7 +10570,7 @@
       </c>
       <c r="E502" t="inlineStr">
         <is>
-          <t>2026-04-05 10:56:03 UTC</t>
+          <t>2026-04-06 08:07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -10621,7 +10621,7 @@
         </is>
       </c>
       <c r="B505" t="n">
-        <v>4635.2</v>
+        <v>757</v>
       </c>
       <c r="C505" t="inlineStr">
         <is>
@@ -10630,7 +10630,7 @@
       </c>
       <c r="E505" t="inlineStr">
         <is>
-          <t>2026-04-05 10:56:35 UTC</t>
+          <t>2026-04-06 08:12:59 UTC</t>
         </is>
       </c>
     </row>
@@ -10861,7 +10861,7 @@
         </is>
       </c>
       <c r="B517" t="n">
-        <v>3171.3</v>
+        <v>754.3</v>
       </c>
       <c r="C517" t="inlineStr">
         <is>
@@ -10870,7 +10870,7 @@
       </c>
       <c r="E517" t="inlineStr">
         <is>
-          <t>2026-04-05 11:03:28 UTC</t>
+          <t>2026-04-06 08:04:33 UTC</t>
         </is>
       </c>
     </row>
@@ -10881,7 +10881,7 @@
         </is>
       </c>
       <c r="B518" t="n">
-        <v>3578.1</v>
+        <v>756.5</v>
       </c>
       <c r="C518" t="inlineStr">
         <is>
@@ -10890,7 +10890,7 @@
       </c>
       <c r="E518" t="inlineStr">
         <is>
-          <t>2026-04-05 11:03:28 UTC</t>
+          <t>2026-04-06 08:12:59 UTC</t>
         </is>
       </c>
     </row>
@@ -10901,7 +10901,7 @@
         </is>
       </c>
       <c r="B519" t="n">
-        <v>2515.2</v>
+        <v>707.7</v>
       </c>
       <c r="C519" t="inlineStr">
         <is>
@@ -10910,7 +10910,7 @@
       </c>
       <c r="E519" t="inlineStr">
         <is>
-          <t>2026-04-06 06:54:04 UTC</t>
+          <t>2026-04-06 09:25:37 UTC</t>
         </is>
       </c>
     </row>
@@ -10941,7 +10941,7 @@
         </is>
       </c>
       <c r="B521" t="n">
-        <v>2794.3</v>
+        <v>1455.1</v>
       </c>
       <c r="C521" t="inlineStr">
         <is>
@@ -10950,7 +10950,7 @@
       </c>
       <c r="E521" t="inlineStr">
         <is>
-          <t>2026-04-05 11:05:09 UTC</t>
+          <t>2026-04-06 09:25:37 UTC</t>
         </is>
       </c>
     </row>
@@ -10961,7 +10961,7 @@
         </is>
       </c>
       <c r="B522" t="n">
-        <v>3134.3</v>
+        <v>1489.6</v>
       </c>
       <c r="C522" t="inlineStr">
         <is>
@@ -10970,7 +10970,7 @@
       </c>
       <c r="E522" t="inlineStr">
         <is>
-          <t>2026-04-05 11:05:09 UTC</t>
+          <t>2026-04-06 09:25:37 UTC</t>
         </is>
       </c>
     </row>
@@ -10981,7 +10981,7 @@
         </is>
       </c>
       <c r="B523" t="n">
-        <v>3390.5</v>
+        <v>3821.6</v>
       </c>
       <c r="C523" t="inlineStr">
         <is>
@@ -10990,7 +10990,7 @@
       </c>
       <c r="E523" t="inlineStr">
         <is>
-          <t>2026-04-05 11:05:09 UTC</t>
+          <t>2026-04-06 08:01:51 UTC</t>
         </is>
       </c>
     </row>
@@ -11081,7 +11081,7 @@
         </is>
       </c>
       <c r="B528" t="n">
-        <v>770.4</v>
+        <v>768</v>
       </c>
       <c r="C528" t="inlineStr">
         <is>
@@ -11090,7 +11090,7 @@
       </c>
       <c r="E528" t="inlineStr">
         <is>
-          <t>2026-04-06 07:15:13 UTC</t>
+          <t>2026-04-06 09:25:37 UTC</t>
         </is>
       </c>
     </row>
@@ -11141,7 +11141,7 @@
         </is>
       </c>
       <c r="B531" t="n">
-        <v>4300.7</v>
+        <v>1914</v>
       </c>
       <c r="C531" t="inlineStr">
         <is>
@@ -11150,7 +11150,7 @@
       </c>
       <c r="E531" t="inlineStr">
         <is>
-          <t>2026-04-05 11:16:29 UTC</t>
+          <t>2026-04-06 09:00:27 UTC</t>
         </is>
       </c>
     </row>
@@ -11161,7 +11161,7 @@
         </is>
       </c>
       <c r="B532" t="n">
-        <v>3480.5</v>
+        <v>4707.6</v>
       </c>
       <c r="C532" t="inlineStr">
         <is>
@@ -11170,7 +11170,7 @@
       </c>
       <c r="E532" t="inlineStr">
         <is>
-          <t>2026-04-06 07:13:50 UTC</t>
+          <t>2026-04-06 07:30:24 UTC</t>
         </is>
       </c>
     </row>
@@ -11301,7 +11301,7 @@
         </is>
       </c>
       <c r="B539" t="n">
-        <v>3303.9</v>
+        <v>2450.2</v>
       </c>
       <c r="C539" t="inlineStr">
         <is>
@@ -11310,7 +11310,7 @@
       </c>
       <c r="E539" t="inlineStr">
         <is>
-          <t>2026-04-06 06:51:21 UTC</t>
+          <t>2026-04-06 09:11:31 UTC</t>
         </is>
       </c>
     </row>
@@ -12141,7 +12141,7 @@
         </is>
       </c>
       <c r="B581" t="n">
-        <v>3734.2</v>
+        <v>915.6</v>
       </c>
       <c r="C581" t="inlineStr">
         <is>
@@ -12150,7 +12150,7 @@
       </c>
       <c r="E581" t="inlineStr">
         <is>
-          <t>2026-04-05 11:31:46 UTC</t>
+          <t>2026-04-06 09:11:31 UTC</t>
         </is>
       </c>
     </row>
@@ -12221,7 +12221,7 @@
         </is>
       </c>
       <c r="B585" t="n">
-        <v>2558.2</v>
+        <v>1290.2</v>
       </c>
       <c r="C585" t="inlineStr">
         <is>
@@ -12230,7 +12230,7 @@
       </c>
       <c r="E585" t="inlineStr">
         <is>
-          <t>2026-04-05 11:38:25 UTC</t>
+          <t>2026-04-06 09:25:37 UTC</t>
         </is>
       </c>
     </row>
@@ -12241,7 +12241,7 @@
         </is>
       </c>
       <c r="B586" t="n">
-        <v>2299.7</v>
+        <v>3637.5</v>
       </c>
       <c r="C586" t="inlineStr">
         <is>
@@ -12250,7 +12250,7 @@
       </c>
       <c r="E586" t="inlineStr">
         <is>
-          <t>2026-04-05 11:38:25 UTC</t>
+          <t>2026-04-06 09:25:37 UTC</t>
         </is>
       </c>
     </row>
@@ -12261,7 +12261,7 @@
         </is>
       </c>
       <c r="B587" t="n">
-        <v>598.3</v>
+        <v>716.7</v>
       </c>
       <c r="C587" t="inlineStr">
         <is>
@@ -12270,7 +12270,7 @@
       </c>
       <c r="E587" t="inlineStr">
         <is>
-          <t>2026-04-06 07:03:40 UTC</t>
+          <t>2026-04-06 07:54:31 UTC</t>
         </is>
       </c>
     </row>
@@ -12281,7 +12281,7 @@
         </is>
       </c>
       <c r="B588" t="n">
-        <v>3635.4</v>
+        <v>62.8</v>
       </c>
       <c r="C588" t="inlineStr">
         <is>
@@ -12290,7 +12290,7 @@
       </c>
       <c r="E588" t="inlineStr">
         <is>
-          <t>2026-04-05 11:38:25 UTC</t>
+          <t>2026-04-06 08:57:08 UTC</t>
         </is>
       </c>
     </row>
@@ -12361,7 +12361,7 @@
         </is>
       </c>
       <c r="B592" t="n">
-        <v>2544.7</v>
+        <v>2034.9</v>
       </c>
       <c r="C592" t="inlineStr">
         <is>
@@ -12370,7 +12370,7 @@
       </c>
       <c r="E592" t="inlineStr">
         <is>
-          <t>2026-04-05 11:38:25 UTC</t>
+          <t>2026-04-06 09:25:37 UTC</t>
         </is>
       </c>
     </row>
@@ -12441,7 +12441,7 @@
         </is>
       </c>
       <c r="B596" t="n">
-        <v>2418</v>
+        <v>1057.4</v>
       </c>
       <c r="C596" t="inlineStr">
         <is>
@@ -12450,7 +12450,7 @@
       </c>
       <c r="E596" t="inlineStr">
         <is>
-          <t>2026-04-05 11:39:10 UTC</t>
+          <t>2026-04-06 08:09:29 UTC</t>
         </is>
       </c>
     </row>
@@ -12481,7 +12481,7 @@
         </is>
       </c>
       <c r="B598" t="n">
-        <v>2608.9</v>
+        <v>837.5</v>
       </c>
       <c r="C598" t="inlineStr">
         <is>
@@ -12490,7 +12490,7 @@
       </c>
       <c r="E598" t="inlineStr">
         <is>
-          <t>2026-04-06 06:37:12 UTC</t>
+          <t>2026-04-06 08:03:11 UTC</t>
         </is>
       </c>
     </row>
@@ -12501,7 +12501,7 @@
         </is>
       </c>
       <c r="B599" t="n">
-        <v>4889.7</v>
+        <v>949.6</v>
       </c>
       <c r="C599" t="inlineStr">
         <is>
@@ -12510,7 +12510,7 @@
       </c>
       <c r="E599" t="inlineStr">
         <is>
-          <t>2026-04-06 06:55:51 UTC</t>
+          <t>2026-04-06 08:03:11 UTC</t>
         </is>
       </c>
     </row>
@@ -12561,7 +12561,7 @@
         </is>
       </c>
       <c r="B602" t="n">
-        <v>2463.9</v>
+        <v>753.9</v>
       </c>
       <c r="C602" t="inlineStr">
         <is>
@@ -12570,7 +12570,7 @@
       </c>
       <c r="E602" t="inlineStr">
         <is>
-          <t>2026-04-05 11:39:10 UTC</t>
+          <t>2026-04-06 08:12:59 UTC</t>
         </is>
       </c>
     </row>
@@ -12621,7 +12621,7 @@
         </is>
       </c>
       <c r="B605" t="n">
-        <v>2438.5</v>
+        <v>1154.7</v>
       </c>
       <c r="C605" t="inlineStr">
         <is>
@@ -12630,7 +12630,7 @@
       </c>
       <c r="E605" t="inlineStr">
         <is>
-          <t>2026-04-05 11:39:48 UTC</t>
+          <t>2026-04-06 09:25:37 UTC</t>
         </is>
       </c>
     </row>
@@ -12641,7 +12641,7 @@
         </is>
       </c>
       <c r="B606" t="n">
-        <v>2339.3</v>
+        <v>1744.3</v>
       </c>
       <c r="C606" t="inlineStr">
         <is>
@@ -12650,7 +12650,7 @@
       </c>
       <c r="E606" t="inlineStr">
         <is>
-          <t>2026-04-05 11:39:48 UTC</t>
+          <t>2026-04-06 09:24:07 UTC</t>
         </is>
       </c>
     </row>
@@ -12661,7 +12661,7 @@
         </is>
       </c>
       <c r="B607" t="n">
-        <v>3822.5</v>
+        <v>3598.4</v>
       </c>
       <c r="C607" t="inlineStr">
         <is>
@@ -12670,7 +12670,7 @@
       </c>
       <c r="E607" t="inlineStr">
         <is>
-          <t>2026-04-05 11:39:48 UTC</t>
+          <t>2026-04-06 09:13:54 UTC</t>
         </is>
       </c>
     </row>
@@ -13221,7 +13221,7 @@
         </is>
       </c>
       <c r="B635" t="n">
-        <v>3826.9</v>
+        <v>3463.7</v>
       </c>
       <c r="C635" t="inlineStr">
         <is>
@@ -13230,7 +13230,7 @@
       </c>
       <c r="E635" t="inlineStr">
         <is>
-          <t>2026-04-05 11:40:16 UTC</t>
+          <t>2026-04-06 08:21:08 UTC</t>
         </is>
       </c>
     </row>
@@ -13301,7 +13301,7 @@
         </is>
       </c>
       <c r="B639" t="n">
-        <v>3151.8</v>
+        <v>763.6</v>
       </c>
       <c r="C639" t="inlineStr">
         <is>
@@ -13310,7 +13310,7 @@
       </c>
       <c r="E639" t="inlineStr">
         <is>
-          <t>2026-04-05 11:47:25 UTC</t>
+          <t>2026-04-06 09:25:37 UTC</t>
         </is>
       </c>
     </row>
@@ -13321,7 +13321,7 @@
         </is>
       </c>
       <c r="B640" t="n">
-        <v>2729.7</v>
+        <v>920.5</v>
       </c>
       <c r="C640" t="inlineStr">
         <is>
@@ -13330,7 +13330,7 @@
       </c>
       <c r="E640" t="inlineStr">
         <is>
-          <t>2026-04-05 11:47:25 UTC</t>
+          <t>2026-04-06 09:24:07 UTC</t>
         </is>
       </c>
     </row>
@@ -13361,7 +13361,7 @@
         </is>
       </c>
       <c r="B642" t="n">
-        <v>2290.5</v>
+        <v>1998.2</v>
       </c>
       <c r="C642" t="inlineStr">
         <is>
@@ -13370,7 +13370,7 @@
       </c>
       <c r="E642" t="inlineStr">
         <is>
-          <t>2026-04-05 11:47:58 UTC</t>
+          <t>2026-04-06 09:25:37 UTC</t>
         </is>
       </c>
     </row>
@@ -13441,7 +13441,7 @@
         </is>
       </c>
       <c r="B646" t="n">
-        <v>2877.4</v>
+        <v>835.6</v>
       </c>
       <c r="C646" t="inlineStr">
         <is>
@@ -13450,7 +13450,7 @@
       </c>
       <c r="E646" t="inlineStr">
         <is>
-          <t>2026-04-05 11:48:31 UTC</t>
+          <t>2026-04-06 09:25:37 UTC</t>
         </is>
       </c>
     </row>
@@ -13841,7 +13841,7 @@
         </is>
       </c>
       <c r="B666" t="n">
-        <v>3458</v>
+        <v>3447.2</v>
       </c>
       <c r="C666" t="inlineStr">
         <is>
@@ -13850,7 +13850,7 @@
       </c>
       <c r="E666" t="inlineStr">
         <is>
-          <t>2026-04-06 07:03:40 UTC</t>
+          <t>2026-04-06 07:17:51 UTC</t>
         </is>
       </c>
     </row>
@@ -13981,7 +13981,7 @@
         </is>
       </c>
       <c r="B673" t="n">
-        <v>3115.2</v>
+        <v>821.2</v>
       </c>
       <c r="C673" t="inlineStr">
         <is>
@@ -13990,7 +13990,7 @@
       </c>
       <c r="E673" t="inlineStr">
         <is>
-          <t>2026-04-05 11:55:44 UTC</t>
+          <t>2026-04-06 08:07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -14421,7 +14421,7 @@
         </is>
       </c>
       <c r="B695" t="n">
-        <v>3656.4</v>
+        <v>2505.7</v>
       </c>
       <c r="C695" t="inlineStr">
         <is>
@@ -14430,7 +14430,7 @@
       </c>
       <c r="E695" t="inlineStr">
         <is>
-          <t>2026-04-05 12:04:49 UTC</t>
+          <t>2026-04-06 09:25:37 UTC</t>
         </is>
       </c>
     </row>
@@ -14441,7 +14441,7 @@
         </is>
       </c>
       <c r="B696" t="n">
-        <v>3551.2</v>
+        <v>4905.6</v>
       </c>
       <c r="C696" t="inlineStr">
         <is>
@@ -14450,7 +14450,7 @@
       </c>
       <c r="E696" t="inlineStr">
         <is>
-          <t>2026-04-05 12:04:49 UTC</t>
+          <t>2026-04-06 09:16:30 UTC</t>
         </is>
       </c>
     </row>
@@ -14621,7 +14621,7 @@
         </is>
       </c>
       <c r="B705" t="n">
-        <v>3330.9</v>
+        <v>3455.1</v>
       </c>
       <c r="C705" t="inlineStr">
         <is>
@@ -14630,7 +14630,7 @@
       </c>
       <c r="E705" t="inlineStr">
         <is>
-          <t>2026-04-05 12:05:12 UTC</t>
+          <t>2026-04-06 09:24:07 UTC</t>
         </is>
       </c>
     </row>
@@ -14761,7 +14761,7 @@
         </is>
       </c>
       <c r="B712" t="n">
-        <v>4512.2</v>
+        <v>1284.3</v>
       </c>
       <c r="C712" t="inlineStr">
         <is>
@@ -14770,7 +14770,7 @@
       </c>
       <c r="E712" t="inlineStr">
         <is>
-          <t>2026-04-05 12:13:55 UTC</t>
+          <t>2026-04-06 09:25:37 UTC</t>
         </is>
       </c>
     </row>
@@ -14801,7 +14801,7 @@
         </is>
       </c>
       <c r="B714" t="n">
-        <v>3021.3</v>
+        <v>4892.7</v>
       </c>
       <c r="C714" t="inlineStr">
         <is>
@@ -14810,7 +14810,7 @@
       </c>
       <c r="E714" t="inlineStr">
         <is>
-          <t>2026-04-05 12:16:23 UTC</t>
+          <t>2026-04-06 08:24:50 UTC</t>
         </is>
       </c>
     </row>
@@ -14821,7 +14821,7 @@
         </is>
       </c>
       <c r="B715" t="n">
-        <v>1032.2</v>
+        <v>785.2</v>
       </c>
       <c r="C715" t="inlineStr">
         <is>
@@ -14830,7 +14830,7 @@
       </c>
       <c r="E715" t="inlineStr">
         <is>
-          <t>2026-04-06 07:13:50 UTC</t>
+          <t>2026-04-06 08:06:15 UTC</t>
         </is>
       </c>
     </row>
@@ -19181,7 +19181,7 @@
         </is>
       </c>
       <c r="B933" t="n">
-        <v>1035</v>
+        <v>919</v>
       </c>
       <c r="C933" t="inlineStr">
         <is>
@@ -19190,7 +19190,7 @@
       </c>
       <c r="E933" t="inlineStr">
         <is>
-          <t>2026-04-06 06:55:51 UTC</t>
+          <t>2026-04-06 09:25:37 UTC</t>
         </is>
       </c>
     </row>
@@ -19401,7 +19401,7 @@
         </is>
       </c>
       <c r="B944" t="n">
-        <v>4727.4</v>
+        <v>3453.9</v>
       </c>
       <c r="C944" t="inlineStr">
         <is>
@@ -19410,7 +19410,7 @@
       </c>
       <c r="E944" t="inlineStr">
         <is>
-          <t>2026-04-05 12:16:49 UTC</t>
+          <t>2026-04-06 08:14:27 UTC</t>
         </is>
       </c>
     </row>
@@ -19761,7 +19761,7 @@
         </is>
       </c>
       <c r="B962" t="n">
-        <v>2116</v>
+        <v>711.8</v>
       </c>
       <c r="C962" t="inlineStr">
         <is>
@@ -19770,7 +19770,7 @@
       </c>
       <c r="E962" t="inlineStr">
         <is>
-          <t>2026-04-05 12:33:08 UTC</t>
+          <t>2026-04-06 08:31:34 UTC</t>
         </is>
       </c>
     </row>
@@ -19801,7 +19801,7 @@
         </is>
       </c>
       <c r="B964" t="n">
-        <v>3979.3</v>
+        <v>1680.7</v>
       </c>
       <c r="C964" t="inlineStr">
         <is>
@@ -19810,7 +19810,7 @@
       </c>
       <c r="E964" t="inlineStr">
         <is>
-          <t>2026-04-05 12:35:37 UTC</t>
+          <t>2026-04-06 07:57:10 UTC</t>
         </is>
       </c>
     </row>
@@ -19821,7 +19821,7 @@
         </is>
       </c>
       <c r="B965" t="n">
-        <v>4264</v>
+        <v>803.5</v>
       </c>
       <c r="C965" t="inlineStr">
         <is>
@@ -19830,7 +19830,7 @@
       </c>
       <c r="E965" t="inlineStr">
         <is>
-          <t>2026-04-05 12:36:08 UTC</t>
+          <t>2026-04-06 08:03:11 UTC</t>
         </is>
       </c>
     </row>
@@ -19841,7 +19841,7 @@
         </is>
       </c>
       <c r="B966" t="n">
-        <v>4397.9</v>
+        <v>2318.4</v>
       </c>
       <c r="C966" t="inlineStr">
         <is>
@@ -19850,7 +19850,7 @@
       </c>
       <c r="E966" t="inlineStr">
         <is>
-          <t>2026-04-05 12:36:08 UTC</t>
+          <t>2026-04-06 08:50:24 UTC</t>
         </is>
       </c>
     </row>
@@ -19861,7 +19861,7 @@
         </is>
       </c>
       <c r="B967" t="n">
-        <v>2941.6</v>
+        <v>754.7</v>
       </c>
       <c r="C967" t="inlineStr">
         <is>
@@ -19870,7 +19870,7 @@
       </c>
       <c r="E967" t="inlineStr">
         <is>
-          <t>2026-04-06 07:12:33 UTC</t>
+          <t>2026-04-06 08:03:11 UTC</t>
         </is>
       </c>
     </row>
@@ -20041,7 +20041,7 @@
         </is>
       </c>
       <c r="B976" t="n">
-        <v>4683.7</v>
+        <v>1137.7</v>
       </c>
       <c r="C976" t="inlineStr">
         <is>
@@ -20050,7 +20050,7 @@
       </c>
       <c r="E976" t="inlineStr">
         <is>
-          <t>2026-04-05 12:36:32 UTC</t>
+          <t>2026-04-06 09:08:54 UTC</t>
         </is>
       </c>
     </row>
@@ -20101,7 +20101,7 @@
         </is>
       </c>
       <c r="B979" t="n">
-        <v>3114.6</v>
+        <v>1983.3</v>
       </c>
       <c r="C979" t="inlineStr">
         <is>
@@ -20110,7 +20110,7 @@
       </c>
       <c r="E979" t="inlineStr">
         <is>
-          <t>2026-04-05 12:44:06 UTC</t>
+          <t>2026-04-06 09:25:37 UTC</t>
         </is>
       </c>
     </row>
@@ -20541,7 +20541,7 @@
         </is>
       </c>
       <c r="B1001" t="n">
-        <v>76</v>
+        <v>90.7</v>
       </c>
       <c r="C1001" t="inlineStr">
         <is>
@@ -20550,7 +20550,7 @@
       </c>
       <c r="E1001" t="inlineStr">
         <is>
-          <t>2026-04-06 07:01:04 UTC</t>
+          <t>2026-04-06 09:11:31 UTC</t>
         </is>
       </c>
     </row>
@@ -20801,7 +20801,7 @@
         </is>
       </c>
       <c r="B1014" t="n">
-        <v>171.8</v>
+        <v>155.2</v>
       </c>
       <c r="C1014" t="inlineStr">
         <is>
@@ -20810,7 +20810,7 @@
       </c>
       <c r="E1014" t="inlineStr">
         <is>
-          <t>2026-04-06 07:01:04 UTC</t>
+          <t>2026-04-06 09:09:56 UTC</t>
         </is>
       </c>
     </row>
@@ -20821,7 +20821,7 @@
         </is>
       </c>
       <c r="B1015" t="n">
-        <v>233.4</v>
+        <v>210.8</v>
       </c>
       <c r="C1015" t="inlineStr">
         <is>
@@ -20830,7 +20830,7 @@
       </c>
       <c r="E1015" t="inlineStr">
         <is>
-          <t>2026-04-06 02:44:39 UTC</t>
+          <t>2026-04-06 09:16:30 UTC</t>
         </is>
       </c>
     </row>
@@ -20881,7 +20881,7 @@
         </is>
       </c>
       <c r="B1018" t="n">
-        <v>3717</v>
+        <v>2851.8</v>
       </c>
       <c r="C1018" t="inlineStr">
         <is>
@@ -20890,7 +20890,7 @@
       </c>
       <c r="E1018" t="inlineStr">
         <is>
-          <t>2026-04-05 13:01:44 UTC</t>
+          <t>2026-04-06 09:25:37 UTC</t>
         </is>
       </c>
     </row>
@@ -20901,7 +20901,7 @@
         </is>
       </c>
       <c r="B1019" t="n">
-        <v>3415.2</v>
+        <v>1012.7</v>
       </c>
       <c r="C1019" t="inlineStr">
         <is>
@@ -20910,7 +20910,7 @@
       </c>
       <c r="E1019" t="inlineStr">
         <is>
-          <t>2026-04-05 13:01:44 UTC</t>
+          <t>2026-04-06 09:24:07 UTC</t>
         </is>
       </c>
     </row>
@@ -20921,7 +20921,7 @@
         </is>
       </c>
       <c r="B1020" t="n">
-        <v>3997.8</v>
+        <v>2221</v>
       </c>
       <c r="C1020" t="inlineStr">
         <is>
@@ -20930,7 +20930,7 @@
       </c>
       <c r="E1020" t="inlineStr">
         <is>
-          <t>2026-04-05 13:01:44 UTC</t>
+          <t>2026-04-06 07:25:19 UTC</t>
         </is>
       </c>
     </row>
@@ -20941,7 +20941,7 @@
         </is>
       </c>
       <c r="B1021" t="n">
-        <v>4687.4</v>
+        <v>3359.9</v>
       </c>
       <c r="C1021" t="inlineStr">
         <is>
@@ -20950,7 +20950,7 @@
       </c>
       <c r="E1021" t="inlineStr">
         <is>
-          <t>2026-04-05 13:01:44 UTC</t>
+          <t>2026-04-06 09:25:37 UTC</t>
         </is>
       </c>
     </row>
@@ -20981,7 +20981,7 @@
         </is>
       </c>
       <c r="B1023" t="n">
-        <v>4897.1</v>
+        <v>896.6</v>
       </c>
       <c r="C1023" t="inlineStr">
         <is>
@@ -20990,7 +20990,7 @@
       </c>
       <c r="E1023" t="inlineStr">
         <is>
-          <t>2026-04-06 07:04:58 UTC</t>
+          <t>2026-04-06 08:07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -21021,7 +21021,7 @@
         </is>
       </c>
       <c r="B1025" t="n">
-        <v>2706.4</v>
+        <v>4068.5</v>
       </c>
       <c r="C1025" t="inlineStr">
         <is>
@@ -21030,7 +21030,7 @@
       </c>
       <c r="E1025" t="inlineStr">
         <is>
-          <t>2026-04-06 06:40:25 UTC</t>
+          <t>2026-04-06 07:58:30 UTC</t>
         </is>
       </c>
     </row>
@@ -21041,7 +21041,7 @@
         </is>
       </c>
       <c r="B1026" t="n">
-        <v>3400.8</v>
+        <v>714.6</v>
       </c>
       <c r="C1026" t="inlineStr">
         <is>
@@ -21050,7 +21050,7 @@
       </c>
       <c r="E1026" t="inlineStr">
         <is>
-          <t>2026-04-05 13:05:38 UTC</t>
+          <t>2026-04-06 08:36:43 UTC</t>
         </is>
       </c>
     </row>
@@ -21101,7 +21101,7 @@
         </is>
       </c>
       <c r="B1029" t="n">
-        <v>3398</v>
+        <v>1760</v>
       </c>
       <c r="C1029" t="inlineStr">
         <is>
@@ -21110,7 +21110,7 @@
       </c>
       <c r="E1029" t="inlineStr">
         <is>
-          <t>2026-04-05 13:05:38 UTC</t>
+          <t>2026-04-06 08:33:36 UTC</t>
         </is>
       </c>
     </row>
@@ -21441,7 +21441,7 @@
         </is>
       </c>
       <c r="B1046" t="n">
-        <v>3657</v>
+        <v>1672.6</v>
       </c>
       <c r="C1046" t="inlineStr">
         <is>
@@ -21450,7 +21450,7 @@
       </c>
       <c r="E1046" t="inlineStr">
         <is>
-          <t>2026-04-05 13:06:19 UTC</t>
+          <t>2026-04-06 07:42:44 UTC</t>
         </is>
       </c>
     </row>
@@ -21541,7 +21541,7 @@
         </is>
       </c>
       <c r="B1051" t="n">
-        <v>4746</v>
+        <v>4256.4</v>
       </c>
       <c r="C1051" t="inlineStr">
         <is>
@@ -21550,7 +21550,7 @@
       </c>
       <c r="E1051" t="inlineStr">
         <is>
-          <t>2026-04-05 13:12:35 UTC</t>
+          <t>2026-04-06 08:48:45 UTC</t>
         </is>
       </c>
     </row>
@@ -21721,7 +21721,7 @@
         </is>
       </c>
       <c r="B1060" t="n">
-        <v>3046.3</v>
+        <v>4938.4</v>
       </c>
       <c r="C1060" t="inlineStr">
         <is>
@@ -21730,7 +21730,7 @@
       </c>
       <c r="E1060" t="inlineStr">
         <is>
-          <t>2026-04-05 13:22:05 UTC</t>
+          <t>2026-04-06 08:12:59 UTC</t>
         </is>
       </c>
     </row>
@@ -21741,7 +21741,7 @@
         </is>
       </c>
       <c r="B1061" t="n">
-        <v>582.9</v>
+        <v>4211.2</v>
       </c>
       <c r="C1061" t="inlineStr">
         <is>
@@ -21750,7 +21750,7 @@
       </c>
       <c r="E1061" t="inlineStr">
         <is>
-          <t>2026-04-06 07:13:50 UTC</t>
+          <t>2026-04-06 07:20:19 UTC</t>
         </is>
       </c>
     </row>
@@ -21761,7 +21761,7 @@
         </is>
       </c>
       <c r="B1062" t="n">
-        <v>4025.4</v>
+        <v>4971.1</v>
       </c>
       <c r="C1062" t="inlineStr">
         <is>
@@ -21770,7 +21770,7 @@
       </c>
       <c r="E1062" t="inlineStr">
         <is>
-          <t>2026-04-05 13:22:05 UTC</t>
+          <t>2026-04-06 07:57:10 UTC</t>
         </is>
       </c>
     </row>
@@ -21801,7 +21801,7 @@
         </is>
       </c>
       <c r="B1064" t="n">
-        <v>3972.7</v>
+        <v>3739.3</v>
       </c>
       <c r="C1064" t="inlineStr">
         <is>
@@ -21810,7 +21810,7 @@
       </c>
       <c r="E1064" t="inlineStr">
         <is>
-          <t>2026-04-05 13:23:10 UTC</t>
+          <t>2026-04-06 08:24:50 UTC</t>
         </is>
       </c>
     </row>
@@ -21821,7 +21821,7 @@
         </is>
       </c>
       <c r="B1065" t="n">
-        <v>3493.6</v>
+        <v>2622.1</v>
       </c>
       <c r="C1065" t="inlineStr">
         <is>
@@ -21830,7 +21830,7 @@
       </c>
       <c r="E1065" t="inlineStr">
         <is>
-          <t>2026-04-05 13:23:10 UTC</t>
+          <t>2026-04-06 08:57:08 UTC</t>
         </is>
       </c>
     </row>
@@ -21841,7 +21841,7 @@
         </is>
       </c>
       <c r="B1066" t="n">
-        <v>3703.2</v>
+        <v>4909.2</v>
       </c>
       <c r="C1066" t="inlineStr">
         <is>
@@ -21850,7 +21850,7 @@
       </c>
       <c r="E1066" t="inlineStr">
         <is>
-          <t>2026-04-05 13:23:10 UTC</t>
+          <t>2026-04-06 08:38:29 UTC</t>
         </is>
       </c>
     </row>
@@ -21941,7 +21941,7 @@
         </is>
       </c>
       <c r="B1071" t="n">
-        <v>3566.4</v>
+        <v>1434.5</v>
       </c>
       <c r="C1071" t="inlineStr">
         <is>
@@ -21950,7 +21950,7 @@
       </c>
       <c r="E1071" t="inlineStr">
         <is>
-          <t>2026-04-05 13:24:19 UTC</t>
+          <t>2026-04-06 09:24:07 UTC</t>
         </is>
       </c>
     </row>
@@ -21961,7 +21961,7 @@
         </is>
       </c>
       <c r="B1072" t="n">
-        <v>2669.4</v>
+        <v>2901.6</v>
       </c>
       <c r="C1072" t="inlineStr">
         <is>
@@ -21970,7 +21970,7 @@
       </c>
       <c r="E1072" t="inlineStr">
         <is>
-          <t>2026-04-05 13:24:19 UTC</t>
+          <t>2026-04-06 08:54:01 UTC</t>
         </is>
       </c>
     </row>
@@ -22121,7 +22121,7 @@
         </is>
       </c>
       <c r="B1080" t="n">
-        <v>213.4</v>
+        <v>3227.6</v>
       </c>
       <c r="C1080" t="inlineStr">
         <is>
@@ -22130,7 +22130,7 @@
       </c>
       <c r="E1080" t="inlineStr">
         <is>
-          <t>2026-04-06 06:33:24 UTC</t>
+          <t>2026-04-06 09:07:33 UTC</t>
         </is>
       </c>
     </row>
@@ -22601,7 +22601,7 @@
         </is>
       </c>
       <c r="B1104" t="n">
-        <v>3299.9</v>
+        <v>4144.4</v>
       </c>
       <c r="C1104" t="inlineStr">
         <is>
@@ -22610,7 +22610,7 @@
       </c>
       <c r="E1104" t="inlineStr">
         <is>
-          <t>2026-04-05 13:31:15 UTC</t>
+          <t>2026-04-06 08:15:52 UTC</t>
         </is>
       </c>
     </row>
@@ -22661,7 +22661,7 @@
         </is>
       </c>
       <c r="B1107" t="n">
-        <v>4489.2</v>
+        <v>4525.2</v>
       </c>
       <c r="C1107" t="inlineStr">
         <is>
@@ -22670,7 +22670,7 @@
       </c>
       <c r="E1107" t="inlineStr">
         <is>
-          <t>2026-04-05 13:32:17 UTC</t>
+          <t>2026-04-06 08:36:43 UTC</t>
         </is>
       </c>
     </row>
@@ -22761,7 +22761,7 @@
         </is>
       </c>
       <c r="B1112" t="n">
-        <v>3737.6</v>
+        <v>2638.2</v>
       </c>
       <c r="C1112" t="inlineStr">
         <is>
@@ -22770,7 +22770,7 @@
       </c>
       <c r="E1112" t="inlineStr">
         <is>
-          <t>2026-04-05 13:32:17 UTC</t>
+          <t>2026-04-06 08:48:45 UTC</t>
         </is>
       </c>
     </row>
@@ -22801,7 +22801,7 @@
         </is>
       </c>
       <c r="B1114" t="n">
-        <v>2620.1</v>
+        <v>1893.7</v>
       </c>
       <c r="C1114" t="inlineStr">
         <is>
@@ -22810,7 +22810,7 @@
       </c>
       <c r="E1114" t="inlineStr">
         <is>
-          <t>2026-04-05 13:32:17 UTC</t>
+          <t>2026-04-06 07:54:31 UTC</t>
         </is>
       </c>
     </row>
@@ -22821,7 +22821,7 @@
         </is>
       </c>
       <c r="B1115" t="n">
-        <v>1939.2</v>
+        <v>1050.9</v>
       </c>
       <c r="C1115" t="inlineStr">
         <is>
@@ -22830,7 +22830,7 @@
       </c>
       <c r="E1115" t="inlineStr">
         <is>
-          <t>2026-04-05 13:35:42 UTC</t>
+          <t>2026-04-06 07:32:41 UTC</t>
         </is>
       </c>
     </row>
@@ -23141,7 +23141,7 @@
         </is>
       </c>
       <c r="B1131" t="n">
-        <v>2523.7</v>
+        <v>1280.9</v>
       </c>
       <c r="C1131" t="inlineStr">
         <is>
@@ -23150,7 +23150,7 @@
       </c>
       <c r="E1131" t="inlineStr">
         <is>
-          <t>2026-04-05 13:45:45 UTC</t>
+          <t>2026-04-06 08:45:32 UTC</t>
         </is>
       </c>
     </row>
@@ -23461,7 +23461,7 @@
         </is>
       </c>
       <c r="B1147" t="n">
-        <v>2777</v>
+        <v>2369.7</v>
       </c>
       <c r="C1147" t="inlineStr">
         <is>
@@ -23470,7 +23470,7 @@
       </c>
       <c r="E1147" t="inlineStr">
         <is>
-          <t>2026-04-05 14:04:32 UTC</t>
+          <t>2026-04-06 09:25:37 UTC</t>
         </is>
       </c>
     </row>
@@ -23481,7 +23481,7 @@
         </is>
       </c>
       <c r="B1148" t="n">
-        <v>2662</v>
+        <v>3474.5</v>
       </c>
       <c r="C1148" t="inlineStr">
         <is>
@@ -23490,7 +23490,7 @@
       </c>
       <c r="E1148" t="inlineStr">
         <is>
-          <t>2026-04-05 14:04:32 UTC</t>
+          <t>2026-04-06 08:06:15 UTC</t>
         </is>
       </c>
     </row>
@@ -23541,7 +23541,7 @@
         </is>
       </c>
       <c r="B1151" t="n">
-        <v>3291.2</v>
+        <v>231</v>
       </c>
       <c r="C1151" t="inlineStr">
         <is>
@@ -23550,7 +23550,7 @@
       </c>
       <c r="E1151" t="inlineStr">
         <is>
-          <t>2026-04-05 14:06:23 UTC</t>
+          <t>2026-04-06 08:55:43 UTC</t>
         </is>
       </c>
     </row>
@@ -23561,7 +23561,7 @@
         </is>
       </c>
       <c r="B1152" t="n">
-        <v>851.5</v>
+        <v>767.8</v>
       </c>
       <c r="C1152" t="inlineStr">
         <is>
@@ -23570,7 +23570,7 @@
       </c>
       <c r="E1152" t="inlineStr">
         <is>
-          <t>2026-04-06 07:12:33 UTC</t>
+          <t>2026-04-06 07:55:52 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>